<commit_message>
fix(parser_docx): handle paragraph-style w:rPr without crashing on qn()
qn() only handles single namespaced tags (it does tag.split(':')), so
passing 'w:pPr/w:rPr' exploded with 'too many values to unpack' on any
DOCX whose paragraph style nests run properties under w:pPr/w:rPr.
Replace the inline path with a _style_rpr() helper that walks the two
levels by hand and falls back to w:rPr for character styles.

Also re-uploads the cleaned-up template xlsx.

Repro file: 'קרוב יותר- דן ואליס.docx' now parses to 92 items and
exports a 81KB PDF end-to-end.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/טבלת ניתוחים ריקה.xlsx
+++ b/טבלת ניתוחים ריקה.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BD053D5-D905-422D-B31F-2AF876CD5A57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD52CFA3-BB28-475A-939C-99BA7CF7B324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -306,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -376,6 +376,18 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
@@ -388,41 +400,32 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="distributed" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="distributed" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -723,7 +726,7 @@
     <col min="3" max="3" width="17.140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="25.85546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="15.28515625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="28.5703125" style="2" customWidth="1"/>
     <col min="7" max="12" width="9" style="2"/>
     <col min="13" max="13" width="23.7109375" style="2" customWidth="1"/>
   </cols>
@@ -741,76 +744,76 @@
       <c r="F1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
     </row>
     <row r="2" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="28" t="s">
+      <c r="B2" s="37"/>
+      <c r="C2" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="32"/>
-      <c r="F2" s="28" t="s">
+      <c r="E2" s="38"/>
+      <c r="F2" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
     </row>
     <row r="3" spans="1:13" ht="111" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
-      <c r="K3" s="27"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="27"/>
+      <c r="A3" s="36"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
     </row>
     <row r="4" spans="1:13" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="38" t="s">
+      <c r="E4" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
-      <c r="M4" s="40"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="34"/>
+      <c r="K4" s="34"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="35"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>

</xml_diff>

<commit_message>
feat: branded UI, dense page layout, blank-row breathing
- Replace pink rectangle + brand text with logo-chubbuck-wide.png
  inside a 33vh magenta hero band (object-fit: cover, pre-padded
  to 5.33:1 so cover never crops the wordmark).
- filler: drop _PRINT_SCALE_PCT 61 -> 55 (template overflows A4
  landscape width at scale 57+, causing one phantom right-overflow
  page per content page).
- filler: HEADER_ROWS_HEIGHT_PT 299.25 -> 324.75 (matches actual
  template R1=52.5 + R2=42 + R3=174 + R4=56.25; previous value
  under-counted page-1 header and orphaned last data row).
- filler: pin ws.print_area = A1:M{last_row} as belt-and-suspenders
  against right/bottom phantom pages.
- filler: _add_breathing_blanks inserts a blank at the top of every
  output and between an opening stage_direction block and the first
  character name.
- Update CLAUDE.md to reflect new constants, print_area rationale,
  hero/logo layout, and breathing-blanks behavior.
</commit_message>
<xml_diff>
--- a/טבלת ניתוחים ריקה.xlsx
+++ b/טבלת ניתוחים ריקה.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD52CFA3-BB28-475A-939C-99BA7CF7B324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{874E4FBB-55E0-485D-B6EC-0E43B2FCDE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -140,16 +140,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="20"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="18"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="20"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -164,7 +164,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0097CC"/>
+        <fgColor rgb="FF6E0134"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -370,24 +370,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
@@ -400,32 +388,44 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="distributed" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="distributed" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="distributed" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="distributed" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,6 +435,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF6E0134"/>
+      <color rgb="FF32539B"/>
       <color rgb="FF0097CC"/>
       <color rgb="FFFF9393"/>
       <color rgb="FF007BA7"/>
@@ -722,16 +724,16 @@
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="62.42578125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="60.85546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="24" style="2" customWidth="1"/>
     <col min="4" max="4" width="25.85546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="15.28515625" style="2" customWidth="1"/>
     <col min="6" max="6" width="28.5703125" style="2" customWidth="1"/>
     <col min="7" max="12" width="9" style="2"/>
-    <col min="13" max="13" width="23.7109375" style="2" customWidth="1"/>
+    <col min="13" max="13" width="21.5703125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="22" t="s">
         <v>4</v>
       </c>
@@ -744,76 +746,76 @@
       <c r="F1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
     </row>
     <row r="2" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="40" t="s">
+      <c r="B2" s="30"/>
+      <c r="C2" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="38"/>
-      <c r="F2" s="32" t="s">
+      <c r="E2" s="33"/>
+      <c r="F2" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
     </row>
     <row r="3" spans="1:13" ht="111" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="36"/>
-      <c r="B3" s="37"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
-      <c r="K3" s="31"/>
-      <c r="L3" s="31"/>
-      <c r="M3" s="31"/>
+      <c r="A3" s="29"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="27"/>
     </row>
     <row r="4" spans="1:13" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="E4" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="35"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
+      <c r="K4" s="40"/>
+      <c r="L4" s="40"/>
+      <c r="M4" s="41"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>

</xml_diff>

<commit_message>
chore: update template + document deploy architecture in CLAUDE.md
- Refresh טבלת ניתוחים ריקה.xlsx with the latest edits. The template
  is bundled into the Lambda image at build time (TEMPLATE_PATH in
  main.py:53), so this commit + deploy is what gets users the new
  version.
- CLAUDE.md: add a Deployment section covering the two-origin
  CloudFront topology (S3 static for /, Lambda for /api/*), the full
  four-step workflow, the diagnostic pointer when the UI doesn't
  match the latest commit, and the scoped OIDC permissions.
</commit_message>
<xml_diff>
--- a/טבלת ניתוחים ריקה.xlsx
+++ b/טבלת ניתוחים ריקה.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{874E4FBB-55E0-485D-B6EC-0E43B2FCDE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6BE2AF6-8C10-41CA-BD42-53455A17AD0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -306,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -368,13 +368,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+      <alignment horizontal="center" vertical="top" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
@@ -385,12 +379,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
@@ -426,6 +414,15 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -723,10 +720,10 @@
   <dimension ref="A1:M173"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="60.85546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="24" style="2" customWidth="1"/>
-    <col min="4" max="4" width="25.85546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="61" style="2" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="23.42578125" style="2" customWidth="1"/>
     <col min="5" max="5" width="15.28515625" style="2" customWidth="1"/>
     <col min="6" max="6" width="28.5703125" style="2" customWidth="1"/>
     <col min="7" max="12" width="9" style="2"/>
@@ -734,88 +731,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="24" t="s">
+      <c r="B1" s="39"/>
+      <c r="C1" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="23"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24" t="s">
+      <c r="D1" s="39"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
     </row>
     <row r="2" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="31" t="s">
+      <c r="B2" s="26"/>
+      <c r="C2" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="33" t="s">
+      <c r="D2" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="33"/>
-      <c r="F2" s="28" t="s">
+      <c r="E2" s="29"/>
+      <c r="F2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
     </row>
     <row r="3" spans="1:13" ht="111" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
-      <c r="K3" s="27"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="27"/>
+      <c r="A3" s="40"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="25"/>
     </row>
     <row r="4" spans="1:13" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="39" t="s">
+      <c r="E4" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
-      <c r="I4" s="40"/>
-      <c r="J4" s="40"/>
-      <c r="K4" s="40"/>
-      <c r="L4" s="40"/>
-      <c r="M4" s="41"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="37"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>

</xml_diff>